<commit_message>
BVS correction, removed subsidy for freight vehicles
</commit_message>
<xml_diff>
--- a/InputData/trans/BVS/BAU Vehicle Subsidy.xlsx
+++ b/InputData/trans/BVS/BAU Vehicle Subsidy.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mary Francis Swint\Vensim\eps-indonesia\InputData\trans\BVS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54B24F7B-31AD-4E8C-BE27-C0BC252DBE4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{857F7253-B37C-4977-AD68-3C85ACD66010}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="36285" yWindow="3990" windowWidth="19200" windowHeight="11205" firstSheet="12" activeTab="15" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38520" yWindow="-5880" windowWidth="38640" windowHeight="21120" firstSheet="5" activeTab="15" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -110,9 +110,6 @@
     <t>Conversion, 2024 USD to 2012 USD</t>
   </si>
   <si>
-    <t>Average vehicle prices</t>
-  </si>
-  <si>
     <t>Rupiah</t>
   </si>
   <si>
@@ -195,6 +192,9 @@
   </si>
   <si>
     <t>hydrogen vehicle</t>
+  </si>
+  <si>
+    <t>Average vehicle prices passenger</t>
   </si>
 </sst>
 </file>
@@ -1033,7 +1033,7 @@
   <sheetData>
     <row r="1" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B1">
         <v>2020</v>
@@ -1131,7 +1131,7 @@
     </row>
     <row r="2" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B2">
         <v>0</v>
@@ -1143,121 +1143,93 @@
         <v>0</v>
       </c>
       <c r="E2">
-        <f>Calculation!$E$2</f>
-        <v>2454.0663430602526</v>
+        <v>0</v>
       </c>
       <c r="F2">
-        <f>Calculation!$E$2</f>
-        <v>2454.0663430602526</v>
+        <v>0</v>
       </c>
       <c r="G2">
-        <f>Calculation!$E$2</f>
-        <v>2454.0663430602526</v>
+        <v>0</v>
       </c>
       <c r="H2">
-        <f>Calculation!$E$2</f>
-        <v>2454.0663430602526</v>
+        <v>0</v>
       </c>
       <c r="I2">
-        <f>Calculation!$E$2</f>
-        <v>2454.0663430602526</v>
+        <v>0</v>
       </c>
       <c r="J2">
-        <f>Calculation!$E$2</f>
-        <v>2454.0663430602526</v>
+        <v>0</v>
       </c>
       <c r="K2">
-        <f>Calculation!$E$2</f>
-        <v>2454.0663430602526</v>
+        <v>0</v>
       </c>
       <c r="L2">
-        <f>Calculation!$E$2</f>
-        <v>2454.0663430602526</v>
+        <v>0</v>
       </c>
       <c r="M2">
-        <f>Calculation!$E$2</f>
-        <v>2454.0663430602526</v>
+        <v>0</v>
       </c>
       <c r="N2">
-        <f>Calculation!$E$2</f>
-        <v>2454.0663430602526</v>
+        <v>0</v>
       </c>
       <c r="O2">
-        <f>Calculation!$E$2</f>
-        <v>2454.0663430602526</v>
+        <v>0</v>
       </c>
       <c r="P2">
-        <f>Calculation!$E$2</f>
-        <v>2454.0663430602526</v>
+        <v>0</v>
       </c>
       <c r="Q2">
-        <f>Calculation!$E$2</f>
-        <v>2454.0663430602526</v>
+        <v>0</v>
       </c>
       <c r="R2">
-        <f>Calculation!$E$2</f>
-        <v>2454.0663430602526</v>
+        <v>0</v>
       </c>
       <c r="S2">
-        <f>Calculation!$E$2</f>
-        <v>2454.0663430602526</v>
+        <v>0</v>
       </c>
       <c r="T2">
-        <f>Calculation!$E$2</f>
-        <v>2454.0663430602526</v>
+        <v>0</v>
       </c>
       <c r="U2">
-        <f>Calculation!$E$2</f>
-        <v>2454.0663430602526</v>
+        <v>0</v>
       </c>
       <c r="V2">
-        <f>Calculation!$E$2</f>
-        <v>2454.0663430602526</v>
+        <v>0</v>
       </c>
       <c r="W2">
-        <f>Calculation!$E$2</f>
-        <v>2454.0663430602526</v>
+        <v>0</v>
       </c>
       <c r="X2">
-        <f>Calculation!$E$2</f>
-        <v>2454.0663430602526</v>
+        <v>0</v>
       </c>
       <c r="Y2">
-        <f>Calculation!$E$2</f>
-        <v>2454.0663430602526</v>
+        <v>0</v>
       </c>
       <c r="Z2">
-        <f>Calculation!$E$2</f>
-        <v>2454.0663430602526</v>
+        <v>0</v>
       </c>
       <c r="AA2">
-        <f>Calculation!$E$2</f>
-        <v>2454.0663430602526</v>
+        <v>0</v>
       </c>
       <c r="AB2">
-        <f>Calculation!$E$2</f>
-        <v>2454.0663430602526</v>
+        <v>0</v>
       </c>
       <c r="AC2">
-        <f>Calculation!$E$2</f>
-        <v>2454.0663430602526</v>
+        <v>0</v>
       </c>
       <c r="AD2">
-        <f>Calculation!$E$2</f>
-        <v>2454.0663430602526</v>
+        <v>0</v>
       </c>
       <c r="AE2">
-        <f>Calculation!$E$2</f>
-        <v>2454.0663430602526</v>
+        <v>0</v>
       </c>
       <c r="AF2">
-        <f>Calculation!$E$2</f>
-        <v>2454.0663430602526</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B3">
         <v>0</v>
@@ -1355,7 +1327,7 @@
     </row>
     <row r="4" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B4">
         <v>0</v>
@@ -1453,7 +1425,7 @@
     </row>
     <row r="5" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B5">
         <v>0</v>
@@ -1551,7 +1523,7 @@
     </row>
     <row r="6" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B6">
         <v>0</v>
@@ -1564,120 +1536,120 @@
       </c>
       <c r="E6">
         <f>E2</f>
-        <v>2454.0663430602526</v>
+        <v>0</v>
       </c>
       <c r="F6">
         <f t="shared" ref="F6:AF6" si="0">F2</f>
-        <v>2454.0663430602526</v>
+        <v>0</v>
       </c>
       <c r="G6">
         <f t="shared" si="0"/>
-        <v>2454.0663430602526</v>
+        <v>0</v>
       </c>
       <c r="H6">
         <f t="shared" si="0"/>
-        <v>2454.0663430602526</v>
+        <v>0</v>
       </c>
       <c r="I6">
         <f t="shared" si="0"/>
-        <v>2454.0663430602526</v>
+        <v>0</v>
       </c>
       <c r="J6">
         <f t="shared" si="0"/>
-        <v>2454.0663430602526</v>
+        <v>0</v>
       </c>
       <c r="K6">
         <f t="shared" si="0"/>
-        <v>2454.0663430602526</v>
+        <v>0</v>
       </c>
       <c r="L6">
         <f t="shared" si="0"/>
-        <v>2454.0663430602526</v>
+        <v>0</v>
       </c>
       <c r="M6">
         <f t="shared" si="0"/>
-        <v>2454.0663430602526</v>
+        <v>0</v>
       </c>
       <c r="N6">
         <f t="shared" si="0"/>
-        <v>2454.0663430602526</v>
+        <v>0</v>
       </c>
       <c r="O6">
         <f t="shared" si="0"/>
-        <v>2454.0663430602526</v>
+        <v>0</v>
       </c>
       <c r="P6">
         <f t="shared" si="0"/>
-        <v>2454.0663430602526</v>
+        <v>0</v>
       </c>
       <c r="Q6">
         <f t="shared" si="0"/>
-        <v>2454.0663430602526</v>
+        <v>0</v>
       </c>
       <c r="R6">
         <f t="shared" si="0"/>
-        <v>2454.0663430602526</v>
+        <v>0</v>
       </c>
       <c r="S6">
         <f t="shared" si="0"/>
-        <v>2454.0663430602526</v>
+        <v>0</v>
       </c>
       <c r="T6">
         <f t="shared" si="0"/>
-        <v>2454.0663430602526</v>
+        <v>0</v>
       </c>
       <c r="U6">
         <f t="shared" si="0"/>
-        <v>2454.0663430602526</v>
+        <v>0</v>
       </c>
       <c r="V6">
         <f t="shared" si="0"/>
-        <v>2454.0663430602526</v>
+        <v>0</v>
       </c>
       <c r="W6">
         <f t="shared" si="0"/>
-        <v>2454.0663430602526</v>
+        <v>0</v>
       </c>
       <c r="X6">
         <f t="shared" si="0"/>
-        <v>2454.0663430602526</v>
+        <v>0</v>
       </c>
       <c r="Y6">
         <f t="shared" si="0"/>
-        <v>2454.0663430602526</v>
+        <v>0</v>
       </c>
       <c r="Z6">
         <f t="shared" si="0"/>
-        <v>2454.0663430602526</v>
+        <v>0</v>
       </c>
       <c r="AA6">
         <f t="shared" si="0"/>
-        <v>2454.0663430602526</v>
+        <v>0</v>
       </c>
       <c r="AB6">
         <f t="shared" si="0"/>
-        <v>2454.0663430602526</v>
+        <v>0</v>
       </c>
       <c r="AC6">
         <f t="shared" si="0"/>
-        <v>2454.0663430602526</v>
+        <v>0</v>
       </c>
       <c r="AD6">
         <f t="shared" si="0"/>
-        <v>2454.0663430602526</v>
+        <v>0</v>
       </c>
       <c r="AE6">
         <f t="shared" si="0"/>
-        <v>2454.0663430602526</v>
+        <v>0</v>
       </c>
       <c r="AF6">
         <f t="shared" si="0"/>
-        <v>2454.0663430602526</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B7">
         <v>0</v>
@@ -1775,7 +1747,7 @@
     </row>
     <row r="8" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B8">
         <v>0</v>
@@ -1788,115 +1760,115 @@
       </c>
       <c r="E8">
         <f>E2</f>
-        <v>2454.0663430602526</v>
+        <v>0</v>
       </c>
       <c r="F8">
         <f t="shared" ref="F8:AF8" si="1">F2</f>
-        <v>2454.0663430602526</v>
+        <v>0</v>
       </c>
       <c r="G8">
         <f t="shared" si="1"/>
-        <v>2454.0663430602526</v>
+        <v>0</v>
       </c>
       <c r="H8">
         <f t="shared" si="1"/>
-        <v>2454.0663430602526</v>
+        <v>0</v>
       </c>
       <c r="I8">
         <f t="shared" si="1"/>
-        <v>2454.0663430602526</v>
+        <v>0</v>
       </c>
       <c r="J8">
         <f t="shared" si="1"/>
-        <v>2454.0663430602526</v>
+        <v>0</v>
       </c>
       <c r="K8">
         <f t="shared" si="1"/>
-        <v>2454.0663430602526</v>
+        <v>0</v>
       </c>
       <c r="L8">
         <f t="shared" si="1"/>
-        <v>2454.0663430602526</v>
+        <v>0</v>
       </c>
       <c r="M8">
         <f t="shared" si="1"/>
-        <v>2454.0663430602526</v>
+        <v>0</v>
       </c>
       <c r="N8">
         <f t="shared" si="1"/>
-        <v>2454.0663430602526</v>
+        <v>0</v>
       </c>
       <c r="O8">
         <f t="shared" si="1"/>
-        <v>2454.0663430602526</v>
+        <v>0</v>
       </c>
       <c r="P8">
         <f t="shared" si="1"/>
-        <v>2454.0663430602526</v>
+        <v>0</v>
       </c>
       <c r="Q8">
         <f t="shared" si="1"/>
-        <v>2454.0663430602526</v>
+        <v>0</v>
       </c>
       <c r="R8">
         <f t="shared" si="1"/>
-        <v>2454.0663430602526</v>
+        <v>0</v>
       </c>
       <c r="S8">
         <f t="shared" si="1"/>
-        <v>2454.0663430602526</v>
+        <v>0</v>
       </c>
       <c r="T8">
         <f t="shared" si="1"/>
-        <v>2454.0663430602526</v>
+        <v>0</v>
       </c>
       <c r="U8">
         <f t="shared" si="1"/>
-        <v>2454.0663430602526</v>
+        <v>0</v>
       </c>
       <c r="V8">
         <f t="shared" si="1"/>
-        <v>2454.0663430602526</v>
+        <v>0</v>
       </c>
       <c r="W8">
         <f t="shared" si="1"/>
-        <v>2454.0663430602526</v>
+        <v>0</v>
       </c>
       <c r="X8">
         <f t="shared" si="1"/>
-        <v>2454.0663430602526</v>
+        <v>0</v>
       </c>
       <c r="Y8">
         <f t="shared" si="1"/>
-        <v>2454.0663430602526</v>
+        <v>0</v>
       </c>
       <c r="Z8">
         <f t="shared" si="1"/>
-        <v>2454.0663430602526</v>
+        <v>0</v>
       </c>
       <c r="AA8">
         <f t="shared" si="1"/>
-        <v>2454.0663430602526</v>
+        <v>0</v>
       </c>
       <c r="AB8">
         <f t="shared" si="1"/>
-        <v>2454.0663430602526</v>
+        <v>0</v>
       </c>
       <c r="AC8">
         <f t="shared" si="1"/>
-        <v>2454.0663430602526</v>
+        <v>0</v>
       </c>
       <c r="AD8">
         <f t="shared" si="1"/>
-        <v>2454.0663430602526</v>
+        <v>0</v>
       </c>
       <c r="AE8">
         <f t="shared" si="1"/>
-        <v>2454.0663430602526</v>
+        <v>0</v>
       </c>
       <c r="AF8">
         <f t="shared" si="1"/>
-        <v>2454.0663430602526</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -1918,7 +1890,7 @@
   <sheetData>
     <row r="1" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B1">
         <v>2020</v>
@@ -2016,7 +1988,7 @@
     </row>
     <row r="2" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B2">
         <v>0</v>
@@ -2028,121 +2000,93 @@
         <v>0</v>
       </c>
       <c r="E2">
-        <f>Calculation!$E$3</f>
-        <v>21858.080788390918</v>
+        <v>0</v>
       </c>
       <c r="F2">
-        <f>Calculation!$E$3</f>
-        <v>21858.080788390918</v>
+        <v>0</v>
       </c>
       <c r="G2">
-        <f>Calculation!$E$3</f>
-        <v>21858.080788390918</v>
+        <v>0</v>
       </c>
       <c r="H2">
-        <f>Calculation!$E$3</f>
-        <v>21858.080788390918</v>
+        <v>0</v>
       </c>
       <c r="I2">
-        <f>Calculation!$E$3</f>
-        <v>21858.080788390918</v>
+        <v>0</v>
       </c>
       <c r="J2">
-        <f>Calculation!$E$3</f>
-        <v>21858.080788390918</v>
+        <v>0</v>
       </c>
       <c r="K2">
-        <f>Calculation!$E$3</f>
-        <v>21858.080788390918</v>
+        <v>0</v>
       </c>
       <c r="L2">
-        <f>Calculation!$E$3</f>
-        <v>21858.080788390918</v>
+        <v>0</v>
       </c>
       <c r="M2">
-        <f>Calculation!$E$3</f>
-        <v>21858.080788390918</v>
+        <v>0</v>
       </c>
       <c r="N2">
-        <f>Calculation!$E$3</f>
-        <v>21858.080788390918</v>
+        <v>0</v>
       </c>
       <c r="O2">
-        <f>Calculation!$E$3</f>
-        <v>21858.080788390918</v>
+        <v>0</v>
       </c>
       <c r="P2">
-        <f>Calculation!$E$3</f>
-        <v>21858.080788390918</v>
+        <v>0</v>
       </c>
       <c r="Q2">
-        <f>Calculation!$E$3</f>
-        <v>21858.080788390918</v>
+        <v>0</v>
       </c>
       <c r="R2">
-        <f>Calculation!$E$3</f>
-        <v>21858.080788390918</v>
+        <v>0</v>
       </c>
       <c r="S2">
-        <f>Calculation!$E$3</f>
-        <v>21858.080788390918</v>
+        <v>0</v>
       </c>
       <c r="T2">
-        <f>Calculation!$E$3</f>
-        <v>21858.080788390918</v>
+        <v>0</v>
       </c>
       <c r="U2">
-        <f>Calculation!$E$3</f>
-        <v>21858.080788390918</v>
+        <v>0</v>
       </c>
       <c r="V2">
-        <f>Calculation!$E$3</f>
-        <v>21858.080788390918</v>
+        <v>0</v>
       </c>
       <c r="W2">
-        <f>Calculation!$E$3</f>
-        <v>21858.080788390918</v>
+        <v>0</v>
       </c>
       <c r="X2">
-        <f>Calculation!$E$3</f>
-        <v>21858.080788390918</v>
+        <v>0</v>
       </c>
       <c r="Y2">
-        <f>Calculation!$E$3</f>
-        <v>21858.080788390918</v>
+        <v>0</v>
       </c>
       <c r="Z2">
-        <f>Calculation!$E$3</f>
-        <v>21858.080788390918</v>
+        <v>0</v>
       </c>
       <c r="AA2">
-        <f>Calculation!$E$3</f>
-        <v>21858.080788390918</v>
+        <v>0</v>
       </c>
       <c r="AB2">
-        <f>Calculation!$E$3</f>
-        <v>21858.080788390918</v>
+        <v>0</v>
       </c>
       <c r="AC2">
-        <f>Calculation!$E$3</f>
-        <v>21858.080788390918</v>
+        <v>0</v>
       </c>
       <c r="AD2">
-        <f>Calculation!$E$3</f>
-        <v>21858.080788390918</v>
+        <v>0</v>
       </c>
       <c r="AE2">
-        <f>Calculation!$E$3</f>
-        <v>21858.080788390918</v>
+        <v>0</v>
       </c>
       <c r="AF2">
-        <f>Calculation!$E$3</f>
-        <v>21858.080788390918</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B3">
         <v>0</v>
@@ -2240,7 +2184,7 @@
     </row>
     <row r="4" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B4">
         <v>0</v>
@@ -2338,7 +2282,7 @@
     </row>
     <row r="5" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B5">
         <v>0</v>
@@ -2436,7 +2380,7 @@
     </row>
     <row r="6" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B6">
         <v>0</v>
@@ -2449,120 +2393,120 @@
       </c>
       <c r="E6">
         <f>E2</f>
-        <v>21858.080788390918</v>
+        <v>0</v>
       </c>
       <c r="F6">
         <f t="shared" ref="F6:AF6" si="0">F2</f>
-        <v>21858.080788390918</v>
+        <v>0</v>
       </c>
       <c r="G6">
         <f t="shared" si="0"/>
-        <v>21858.080788390918</v>
+        <v>0</v>
       </c>
       <c r="H6">
         <f t="shared" si="0"/>
-        <v>21858.080788390918</v>
+        <v>0</v>
       </c>
       <c r="I6">
         <f t="shared" si="0"/>
-        <v>21858.080788390918</v>
+        <v>0</v>
       </c>
       <c r="J6">
         <f t="shared" si="0"/>
-        <v>21858.080788390918</v>
+        <v>0</v>
       </c>
       <c r="K6">
         <f t="shared" si="0"/>
-        <v>21858.080788390918</v>
+        <v>0</v>
       </c>
       <c r="L6">
         <f t="shared" si="0"/>
-        <v>21858.080788390918</v>
+        <v>0</v>
       </c>
       <c r="M6">
         <f t="shared" si="0"/>
-        <v>21858.080788390918</v>
+        <v>0</v>
       </c>
       <c r="N6">
         <f t="shared" si="0"/>
-        <v>21858.080788390918</v>
+        <v>0</v>
       </c>
       <c r="O6">
         <f t="shared" si="0"/>
-        <v>21858.080788390918</v>
+        <v>0</v>
       </c>
       <c r="P6">
         <f t="shared" si="0"/>
-        <v>21858.080788390918</v>
+        <v>0</v>
       </c>
       <c r="Q6">
         <f t="shared" si="0"/>
-        <v>21858.080788390918</v>
+        <v>0</v>
       </c>
       <c r="R6">
         <f t="shared" si="0"/>
-        <v>21858.080788390918</v>
+        <v>0</v>
       </c>
       <c r="S6">
         <f t="shared" si="0"/>
-        <v>21858.080788390918</v>
+        <v>0</v>
       </c>
       <c r="T6">
         <f t="shared" si="0"/>
-        <v>21858.080788390918</v>
+        <v>0</v>
       </c>
       <c r="U6">
         <f t="shared" si="0"/>
-        <v>21858.080788390918</v>
+        <v>0</v>
       </c>
       <c r="V6">
         <f t="shared" si="0"/>
-        <v>21858.080788390918</v>
+        <v>0</v>
       </c>
       <c r="W6">
         <f t="shared" si="0"/>
-        <v>21858.080788390918</v>
+        <v>0</v>
       </c>
       <c r="X6">
         <f t="shared" si="0"/>
-        <v>21858.080788390918</v>
+        <v>0</v>
       </c>
       <c r="Y6">
         <f t="shared" si="0"/>
-        <v>21858.080788390918</v>
+        <v>0</v>
       </c>
       <c r="Z6">
         <f t="shared" si="0"/>
-        <v>21858.080788390918</v>
+        <v>0</v>
       </c>
       <c r="AA6">
         <f t="shared" si="0"/>
-        <v>21858.080788390918</v>
+        <v>0</v>
       </c>
       <c r="AB6">
         <f t="shared" si="0"/>
-        <v>21858.080788390918</v>
+        <v>0</v>
       </c>
       <c r="AC6">
         <f t="shared" si="0"/>
-        <v>21858.080788390918</v>
+        <v>0</v>
       </c>
       <c r="AD6">
         <f t="shared" si="0"/>
-        <v>21858.080788390918</v>
+        <v>0</v>
       </c>
       <c r="AE6">
         <f t="shared" si="0"/>
-        <v>21858.080788390918</v>
+        <v>0</v>
       </c>
       <c r="AF6">
         <f t="shared" si="0"/>
-        <v>21858.080788390918</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B7">
         <v>0</v>
@@ -2660,7 +2604,7 @@
     </row>
     <row r="8" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B8">
         <v>0</v>
@@ -2673,115 +2617,115 @@
       </c>
       <c r="E8">
         <f>E2</f>
-        <v>21858.080788390918</v>
+        <v>0</v>
       </c>
       <c r="F8">
         <f t="shared" ref="F8:AF8" si="1">F2</f>
-        <v>21858.080788390918</v>
+        <v>0</v>
       </c>
       <c r="G8">
         <f t="shared" si="1"/>
-        <v>21858.080788390918</v>
+        <v>0</v>
       </c>
       <c r="H8">
         <f t="shared" si="1"/>
-        <v>21858.080788390918</v>
+        <v>0</v>
       </c>
       <c r="I8">
         <f t="shared" si="1"/>
-        <v>21858.080788390918</v>
+        <v>0</v>
       </c>
       <c r="J8">
         <f t="shared" si="1"/>
-        <v>21858.080788390918</v>
+        <v>0</v>
       </c>
       <c r="K8">
         <f t="shared" si="1"/>
-        <v>21858.080788390918</v>
+        <v>0</v>
       </c>
       <c r="L8">
         <f t="shared" si="1"/>
-        <v>21858.080788390918</v>
+        <v>0</v>
       </c>
       <c r="M8">
         <f t="shared" si="1"/>
-        <v>21858.080788390918</v>
+        <v>0</v>
       </c>
       <c r="N8">
         <f t="shared" si="1"/>
-        <v>21858.080788390918</v>
+        <v>0</v>
       </c>
       <c r="O8">
         <f t="shared" si="1"/>
-        <v>21858.080788390918</v>
+        <v>0</v>
       </c>
       <c r="P8">
         <f t="shared" si="1"/>
-        <v>21858.080788390918</v>
+        <v>0</v>
       </c>
       <c r="Q8">
         <f t="shared" si="1"/>
-        <v>21858.080788390918</v>
+        <v>0</v>
       </c>
       <c r="R8">
         <f t="shared" si="1"/>
-        <v>21858.080788390918</v>
+        <v>0</v>
       </c>
       <c r="S8">
         <f t="shared" si="1"/>
-        <v>21858.080788390918</v>
+        <v>0</v>
       </c>
       <c r="T8">
         <f t="shared" si="1"/>
-        <v>21858.080788390918</v>
+        <v>0</v>
       </c>
       <c r="U8">
         <f t="shared" si="1"/>
-        <v>21858.080788390918</v>
+        <v>0</v>
       </c>
       <c r="V8">
         <f t="shared" si="1"/>
-        <v>21858.080788390918</v>
+        <v>0</v>
       </c>
       <c r="W8">
         <f t="shared" si="1"/>
-        <v>21858.080788390918</v>
+        <v>0</v>
       </c>
       <c r="X8">
         <f t="shared" si="1"/>
-        <v>21858.080788390918</v>
+        <v>0</v>
       </c>
       <c r="Y8">
         <f t="shared" si="1"/>
-        <v>21858.080788390918</v>
+        <v>0</v>
       </c>
       <c r="Z8">
         <f t="shared" si="1"/>
-        <v>21858.080788390918</v>
+        <v>0</v>
       </c>
       <c r="AA8">
         <f t="shared" si="1"/>
-        <v>21858.080788390918</v>
+        <v>0</v>
       </c>
       <c r="AB8">
         <f t="shared" si="1"/>
-        <v>21858.080788390918</v>
+        <v>0</v>
       </c>
       <c r="AC8">
         <f t="shared" si="1"/>
-        <v>21858.080788390918</v>
+        <v>0</v>
       </c>
       <c r="AD8">
         <f t="shared" si="1"/>
-        <v>21858.080788390918</v>
+        <v>0</v>
       </c>
       <c r="AE8">
         <f t="shared" si="1"/>
-        <v>21858.080788390918</v>
+        <v>0</v>
       </c>
       <c r="AF8">
         <f t="shared" si="1"/>
-        <v>21858.080788390918</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -2802,7 +2746,7 @@
   <sheetData>
     <row r="1" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B1">
         <v>2020</v>
@@ -2900,7 +2844,7 @@
     </row>
     <row r="2" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B2">
         <v>0</v>
@@ -2998,7 +2942,7 @@
     </row>
     <row r="3" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B3">
         <v>0</v>
@@ -3096,7 +3040,7 @@
     </row>
     <row r="4" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B4">
         <v>0</v>
@@ -3194,7 +3138,7 @@
     </row>
     <row r="5" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B5">
         <v>0</v>
@@ -3292,7 +3236,7 @@
     </row>
     <row r="6" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B6">
         <v>0</v>
@@ -3390,7 +3334,7 @@
     </row>
     <row r="7" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B7">
         <v>0</v>
@@ -3488,7 +3432,7 @@
     </row>
     <row r="8" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B8">
         <v>0</v>
@@ -3602,7 +3546,7 @@
   <sheetData>
     <row r="1" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B1">
         <v>2020</v>
@@ -3700,7 +3644,7 @@
     </row>
     <row r="2" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B2">
         <v>0</v>
@@ -3798,7 +3742,7 @@
     </row>
     <row r="3" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B3">
         <v>0</v>
@@ -3896,7 +3840,7 @@
     </row>
     <row r="4" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B4">
         <v>0</v>
@@ -3994,7 +3938,7 @@
     </row>
     <row r="5" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B5">
         <v>0</v>
@@ -4092,7 +4036,7 @@
     </row>
     <row r="6" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B6">
         <v>0</v>
@@ -4190,7 +4134,7 @@
     </row>
     <row r="7" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B7">
         <v>0</v>
@@ -4288,7 +4232,7 @@
     </row>
     <row r="8" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B8">
         <v>0</v>
@@ -4402,7 +4346,7 @@
   <sheetData>
     <row r="1" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B1">
         <v>2020</v>
@@ -4500,7 +4444,7 @@
     </row>
     <row r="2" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B2">
         <v>0</v>
@@ -4598,7 +4542,7 @@
     </row>
     <row r="3" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B3">
         <v>0</v>
@@ -4696,7 +4640,7 @@
     </row>
     <row r="4" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B4">
         <v>0</v>
@@ -4794,7 +4738,7 @@
     </row>
     <row r="5" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B5">
         <v>0</v>
@@ -4892,7 +4836,7 @@
     </row>
     <row r="6" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B6">
         <v>0</v>
@@ -4990,7 +4934,7 @@
     </row>
     <row r="7" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B7">
         <v>0</v>
@@ -5088,7 +5032,7 @@
     </row>
     <row r="8" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B8">
         <v>0</v>
@@ -5202,7 +5146,7 @@
   <sheetData>
     <row r="1" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B1">
         <v>2020</v>
@@ -5300,7 +5244,7 @@
     </row>
     <row r="2" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B2">
         <v>0</v>
@@ -5312,121 +5256,93 @@
         <v>0</v>
       </c>
       <c r="E2">
-        <f>Calculation!$E$4</f>
-        <v>339.33021860220532</v>
+        <v>0</v>
       </c>
       <c r="F2">
-        <f>Calculation!$E$4</f>
-        <v>339.33021860220532</v>
+        <v>0</v>
       </c>
       <c r="G2">
-        <f>Calculation!$E$4</f>
-        <v>339.33021860220532</v>
+        <v>0</v>
       </c>
       <c r="H2">
-        <f>Calculation!$E$4</f>
-        <v>339.33021860220532</v>
+        <v>0</v>
       </c>
       <c r="I2">
-        <f>Calculation!$E$4</f>
-        <v>339.33021860220532</v>
+        <v>0</v>
       </c>
       <c r="J2">
-        <f>Calculation!$E$4</f>
-        <v>339.33021860220532</v>
+        <v>0</v>
       </c>
       <c r="K2">
-        <f>Calculation!$E$4</f>
-        <v>339.33021860220532</v>
+        <v>0</v>
       </c>
       <c r="L2">
-        <f>Calculation!$E$4</f>
-        <v>339.33021860220532</v>
+        <v>0</v>
       </c>
       <c r="M2">
-        <f>Calculation!$E$4</f>
-        <v>339.33021860220532</v>
+        <v>0</v>
       </c>
       <c r="N2">
-        <f>Calculation!$E$4</f>
-        <v>339.33021860220532</v>
+        <v>0</v>
       </c>
       <c r="O2">
-        <f>Calculation!$E$4</f>
-        <v>339.33021860220532</v>
+        <v>0</v>
       </c>
       <c r="P2">
-        <f>Calculation!$E$4</f>
-        <v>339.33021860220532</v>
+        <v>0</v>
       </c>
       <c r="Q2">
-        <f>Calculation!$E$4</f>
-        <v>339.33021860220532</v>
+        <v>0</v>
       </c>
       <c r="R2">
-        <f>Calculation!$E$4</f>
-        <v>339.33021860220532</v>
+        <v>0</v>
       </c>
       <c r="S2">
-        <f>Calculation!$E$4</f>
-        <v>339.33021860220532</v>
+        <v>0</v>
       </c>
       <c r="T2">
-        <f>Calculation!$E$4</f>
-        <v>339.33021860220532</v>
+        <v>0</v>
       </c>
       <c r="U2">
-        <f>Calculation!$E$4</f>
-        <v>339.33021860220532</v>
+        <v>0</v>
       </c>
       <c r="V2">
-        <f>Calculation!$E$4</f>
-        <v>339.33021860220532</v>
+        <v>0</v>
       </c>
       <c r="W2">
-        <f>Calculation!$E$4</f>
-        <v>339.33021860220532</v>
+        <v>0</v>
       </c>
       <c r="X2">
-        <f>Calculation!$E$4</f>
-        <v>339.33021860220532</v>
+        <v>0</v>
       </c>
       <c r="Y2">
-        <f>Calculation!$E$4</f>
-        <v>339.33021860220532</v>
+        <v>0</v>
       </c>
       <c r="Z2">
-        <f>Calculation!$E$4</f>
-        <v>339.33021860220532</v>
+        <v>0</v>
       </c>
       <c r="AA2">
-        <f>Calculation!$E$4</f>
-        <v>339.33021860220532</v>
+        <v>0</v>
       </c>
       <c r="AB2">
-        <f>Calculation!$E$4</f>
-        <v>339.33021860220532</v>
+        <v>0</v>
       </c>
       <c r="AC2">
-        <f>Calculation!$E$4</f>
-        <v>339.33021860220532</v>
+        <v>0</v>
       </c>
       <c r="AD2">
-        <f>Calculation!$E$4</f>
-        <v>339.33021860220532</v>
+        <v>0</v>
       </c>
       <c r="AE2">
-        <f>Calculation!$E$4</f>
-        <v>339.33021860220532</v>
+        <v>0</v>
       </c>
       <c r="AF2">
-        <f>Calculation!$E$4</f>
-        <v>339.33021860220532</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B3">
         <v>0</v>
@@ -5524,7 +5440,7 @@
     </row>
     <row r="4" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B4">
         <v>0</v>
@@ -5622,7 +5538,7 @@
     </row>
     <row r="5" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B5">
         <v>0</v>
@@ -5720,7 +5636,7 @@
     </row>
     <row r="6" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B6">
         <v>0</v>
@@ -5733,120 +5649,120 @@
       </c>
       <c r="E6">
         <f>E2</f>
-        <v>339.33021860220532</v>
+        <v>0</v>
       </c>
       <c r="F6">
         <f t="shared" ref="F6:AF6" si="0">F2</f>
-        <v>339.33021860220532</v>
+        <v>0</v>
       </c>
       <c r="G6">
         <f t="shared" si="0"/>
-        <v>339.33021860220532</v>
+        <v>0</v>
       </c>
       <c r="H6">
         <f t="shared" si="0"/>
-        <v>339.33021860220532</v>
+        <v>0</v>
       </c>
       <c r="I6">
         <f t="shared" si="0"/>
-        <v>339.33021860220532</v>
+        <v>0</v>
       </c>
       <c r="J6">
         <f t="shared" si="0"/>
-        <v>339.33021860220532</v>
+        <v>0</v>
       </c>
       <c r="K6">
         <f t="shared" si="0"/>
-        <v>339.33021860220532</v>
+        <v>0</v>
       </c>
       <c r="L6">
         <f t="shared" si="0"/>
-        <v>339.33021860220532</v>
+        <v>0</v>
       </c>
       <c r="M6">
         <f t="shared" si="0"/>
-        <v>339.33021860220532</v>
+        <v>0</v>
       </c>
       <c r="N6">
         <f t="shared" si="0"/>
-        <v>339.33021860220532</v>
+        <v>0</v>
       </c>
       <c r="O6">
         <f t="shared" si="0"/>
-        <v>339.33021860220532</v>
+        <v>0</v>
       </c>
       <c r="P6">
         <f t="shared" si="0"/>
-        <v>339.33021860220532</v>
+        <v>0</v>
       </c>
       <c r="Q6">
         <f t="shared" si="0"/>
-        <v>339.33021860220532</v>
+        <v>0</v>
       </c>
       <c r="R6">
         <f t="shared" si="0"/>
-        <v>339.33021860220532</v>
+        <v>0</v>
       </c>
       <c r="S6">
         <f t="shared" si="0"/>
-        <v>339.33021860220532</v>
+        <v>0</v>
       </c>
       <c r="T6">
         <f t="shared" si="0"/>
-        <v>339.33021860220532</v>
+        <v>0</v>
       </c>
       <c r="U6">
         <f t="shared" si="0"/>
-        <v>339.33021860220532</v>
+        <v>0</v>
       </c>
       <c r="V6">
         <f t="shared" si="0"/>
-        <v>339.33021860220532</v>
+        <v>0</v>
       </c>
       <c r="W6">
         <f t="shared" si="0"/>
-        <v>339.33021860220532</v>
+        <v>0</v>
       </c>
       <c r="X6">
         <f t="shared" si="0"/>
-        <v>339.33021860220532</v>
+        <v>0</v>
       </c>
       <c r="Y6">
         <f t="shared" si="0"/>
-        <v>339.33021860220532</v>
+        <v>0</v>
       </c>
       <c r="Z6">
         <f t="shared" si="0"/>
-        <v>339.33021860220532</v>
+        <v>0</v>
       </c>
       <c r="AA6">
         <f t="shared" si="0"/>
-        <v>339.33021860220532</v>
+        <v>0</v>
       </c>
       <c r="AB6">
         <f t="shared" si="0"/>
-        <v>339.33021860220532</v>
+        <v>0</v>
       </c>
       <c r="AC6">
         <f t="shared" si="0"/>
-        <v>339.33021860220532</v>
+        <v>0</v>
       </c>
       <c r="AD6">
         <f t="shared" si="0"/>
-        <v>339.33021860220532</v>
+        <v>0</v>
       </c>
       <c r="AE6">
         <f t="shared" si="0"/>
-        <v>339.33021860220532</v>
+        <v>0</v>
       </c>
       <c r="AF6">
         <f t="shared" si="0"/>
-        <v>339.33021860220532</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B7">
         <v>0</v>
@@ -5944,7 +5860,7 @@
     </row>
     <row r="8" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B8">
         <v>0</v>
@@ -5957,115 +5873,115 @@
       </c>
       <c r="E8">
         <f>E2</f>
-        <v>339.33021860220532</v>
+        <v>0</v>
       </c>
       <c r="F8">
         <f t="shared" ref="F8:AF8" si="1">F2</f>
-        <v>339.33021860220532</v>
+        <v>0</v>
       </c>
       <c r="G8">
         <f t="shared" si="1"/>
-        <v>339.33021860220532</v>
+        <v>0</v>
       </c>
       <c r="H8">
         <f t="shared" si="1"/>
-        <v>339.33021860220532</v>
+        <v>0</v>
       </c>
       <c r="I8">
         <f t="shared" si="1"/>
-        <v>339.33021860220532</v>
+        <v>0</v>
       </c>
       <c r="J8">
         <f t="shared" si="1"/>
-        <v>339.33021860220532</v>
+        <v>0</v>
       </c>
       <c r="K8">
         <f t="shared" si="1"/>
-        <v>339.33021860220532</v>
+        <v>0</v>
       </c>
       <c r="L8">
         <f t="shared" si="1"/>
-        <v>339.33021860220532</v>
+        <v>0</v>
       </c>
       <c r="M8">
         <f t="shared" si="1"/>
-        <v>339.33021860220532</v>
+        <v>0</v>
       </c>
       <c r="N8">
         <f t="shared" si="1"/>
-        <v>339.33021860220532</v>
+        <v>0</v>
       </c>
       <c r="O8">
         <f t="shared" si="1"/>
-        <v>339.33021860220532</v>
+        <v>0</v>
       </c>
       <c r="P8">
         <f t="shared" si="1"/>
-        <v>339.33021860220532</v>
+        <v>0</v>
       </c>
       <c r="Q8">
         <f t="shared" si="1"/>
-        <v>339.33021860220532</v>
+        <v>0</v>
       </c>
       <c r="R8">
         <f t="shared" si="1"/>
-        <v>339.33021860220532</v>
+        <v>0</v>
       </c>
       <c r="S8">
         <f t="shared" si="1"/>
-        <v>339.33021860220532</v>
+        <v>0</v>
       </c>
       <c r="T8">
         <f t="shared" si="1"/>
-        <v>339.33021860220532</v>
+        <v>0</v>
       </c>
       <c r="U8">
         <f t="shared" si="1"/>
-        <v>339.33021860220532</v>
+        <v>0</v>
       </c>
       <c r="V8">
         <f t="shared" si="1"/>
-        <v>339.33021860220532</v>
+        <v>0</v>
       </c>
       <c r="W8">
         <f t="shared" si="1"/>
-        <v>339.33021860220532</v>
+        <v>0</v>
       </c>
       <c r="X8">
         <f t="shared" si="1"/>
-        <v>339.33021860220532</v>
+        <v>0</v>
       </c>
       <c r="Y8">
         <f t="shared" si="1"/>
-        <v>339.33021860220532</v>
+        <v>0</v>
       </c>
       <c r="Z8">
         <f t="shared" si="1"/>
-        <v>339.33021860220532</v>
+        <v>0</v>
       </c>
       <c r="AA8">
         <f t="shared" si="1"/>
-        <v>339.33021860220532</v>
+        <v>0</v>
       </c>
       <c r="AB8">
         <f t="shared" si="1"/>
-        <v>339.33021860220532</v>
+        <v>0</v>
       </c>
       <c r="AC8">
         <f t="shared" si="1"/>
-        <v>339.33021860220532</v>
+        <v>0</v>
       </c>
       <c r="AD8">
         <f t="shared" si="1"/>
-        <v>339.33021860220532</v>
+        <v>0</v>
       </c>
       <c r="AE8">
         <f t="shared" si="1"/>
-        <v>339.33021860220532</v>
+        <v>0</v>
       </c>
       <c r="AF8">
         <f t="shared" si="1"/>
-        <v>339.33021860220532</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -6083,24 +5999,24 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B1" t="s">
         <v>19</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>20</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>21</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>22</v>
-      </c>
-      <c r="E1" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B2">
         <f>617.5*10^6</f>
@@ -6121,7 +6037,7 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B3" s="20">
         <v>5500000000</v>
@@ -6141,7 +6057,7 @@
     </row>
     <row r="4" spans="1:9" ht="27.5" x14ac:dyDescent="1.1499999999999999">
       <c r="A4" s="6" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B4" s="13">
         <v>21275000</v>
@@ -6208,7 +6124,7 @@
         <v>0.11</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C9" s="6"/>
       <c r="D9" s="6"/>
@@ -6237,7 +6153,7 @@
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A11" s="6" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B11" s="6">
         <v>1100</v>
@@ -6255,7 +6171,7 @@
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A12" s="6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B12" s="6">
         <v>100</v>
@@ -6273,7 +6189,7 @@
     </row>
     <row r="13" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A13" s="6" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B13" s="9">
         <v>9.01E-2</v>
@@ -6311,7 +6227,7 @@
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A16" s="6" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B16" s="6"/>
       <c r="C16" s="6"/>
@@ -6323,13 +6239,13 @@
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A17" s="10" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B17" s="11">
         <v>9.01E-2</v>
       </c>
       <c r="C17" s="12" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D17" s="6"/>
       <c r="E17" s="6"/>
@@ -6339,13 +6255,13 @@
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A18" s="10" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B18" s="11">
         <v>9.01E-2</v>
       </c>
       <c r="C18" s="12" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D18" s="6"/>
       <c r="E18" s="6"/>
@@ -6355,13 +6271,13 @@
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A19" s="10" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B19" s="11">
         <v>0.36159999999999998</v>
       </c>
       <c r="C19" s="12" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D19" s="6"/>
       <c r="E19" s="6"/>
@@ -6381,10 +6297,10 @@
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A21" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="B21" s="6" t="s">
         <v>38</v>
-      </c>
-      <c r="B21" s="6" t="s">
-        <v>39</v>
       </c>
       <c r="C21" s="6"/>
       <c r="D21" s="6"/>
@@ -16236,7 +16152,7 @@
   <sheetData>
     <row r="1" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B1">
         <v>2020</v>
@@ -16334,7 +16250,7 @@
     </row>
     <row r="2" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B2" s="5">
         <v>0</v>
@@ -16460,7 +16376,7 @@
     </row>
     <row r="3" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B3" s="5">
         <v>0</v>
@@ -16558,7 +16474,7 @@
     </row>
     <row r="4" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B4" s="5">
         <v>0</v>
@@ -16656,7 +16572,7 @@
     </row>
     <row r="5" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B5" s="5">
         <v>0</v>
@@ -16754,7 +16670,7 @@
     </row>
     <row r="6" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B6" s="5">
         <v>0</v>
@@ -16880,7 +16796,7 @@
     </row>
     <row r="7" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B7" s="5">
         <v>0</v>
@@ -16978,7 +16894,7 @@
     </row>
     <row r="8" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B8" s="5">
         <v>0</v>
@@ -17121,7 +17037,7 @@
   <sheetData>
     <row r="1" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B1">
         <v>2020</v>
@@ -17219,7 +17135,7 @@
     </row>
     <row r="2" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B2">
         <v>0</v>
@@ -17345,7 +17261,7 @@
     </row>
     <row r="3" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B3">
         <v>0</v>
@@ -17443,7 +17359,7 @@
     </row>
     <row r="4" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B4">
         <v>0</v>
@@ -17541,7 +17457,7 @@
     </row>
     <row r="5" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B5">
         <v>0</v>
@@ -17639,7 +17555,7 @@
     </row>
     <row r="6" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B6">
         <v>0</v>
@@ -17765,7 +17681,7 @@
     </row>
     <row r="7" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B7">
         <v>0</v>
@@ -17863,7 +17779,7 @@
     </row>
     <row r="8" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B8">
         <v>0</v>
@@ -18005,7 +17921,7 @@
   <sheetData>
     <row r="1" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B1">
         <v>2020</v>
@@ -18103,7 +18019,7 @@
     </row>
     <row r="2" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B2">
         <v>0</v>
@@ -18201,7 +18117,7 @@
     </row>
     <row r="3" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B3">
         <v>0</v>
@@ -18299,7 +18215,7 @@
     </row>
     <row r="4" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B4">
         <v>0</v>
@@ -18397,7 +18313,7 @@
     </row>
     <row r="5" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B5">
         <v>0</v>
@@ -18495,7 +18411,7 @@
     </row>
     <row r="6" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B6">
         <v>0</v>
@@ -18593,7 +18509,7 @@
     </row>
     <row r="7" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B7">
         <v>0</v>
@@ -18691,7 +18607,7 @@
     </row>
     <row r="8" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B8">
         <v>0</v>
@@ -18805,7 +18721,7 @@
   <sheetData>
     <row r="1" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B1">
         <v>2020</v>
@@ -18903,7 +18819,7 @@
     </row>
     <row r="2" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B2">
         <v>0</v>
@@ -19001,7 +18917,7 @@
     </row>
     <row r="3" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B3">
         <v>0</v>
@@ -19099,7 +19015,7 @@
     </row>
     <row r="4" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B4">
         <v>0</v>
@@ -19197,7 +19113,7 @@
     </row>
     <row r="5" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B5">
         <v>0</v>
@@ -19295,7 +19211,7 @@
     </row>
     <row r="6" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B6">
         <v>0</v>
@@ -19393,7 +19309,7 @@
     </row>
     <row r="7" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B7">
         <v>0</v>
@@ -19491,7 +19407,7 @@
     </row>
     <row r="8" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B8">
         <v>0</v>
@@ -19605,7 +19521,7 @@
   <sheetData>
     <row r="1" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B1">
         <v>2020</v>
@@ -19703,7 +19619,7 @@
     </row>
     <row r="2" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B2">
         <v>0</v>
@@ -19801,7 +19717,7 @@
     </row>
     <row r="3" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B3">
         <v>0</v>
@@ -19899,7 +19815,7 @@
     </row>
     <row r="4" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B4">
         <v>0</v>
@@ -19997,7 +19913,7 @@
     </row>
     <row r="5" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B5">
         <v>0</v>
@@ -20095,7 +20011,7 @@
     </row>
     <row r="6" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B6">
         <v>0</v>
@@ -20193,7 +20109,7 @@
     </row>
     <row r="7" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B7">
         <v>0</v>
@@ -20291,7 +20207,7 @@
     </row>
     <row r="8" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B8">
         <v>0</v>
@@ -20405,7 +20321,7 @@
   <sheetData>
     <row r="1" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B1">
         <v>2020</v>
@@ -20503,7 +20419,7 @@
     </row>
     <row r="2" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B2">
         <f>Calculation!$E$4</f>
@@ -20632,7 +20548,7 @@
     </row>
     <row r="3" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B3">
         <v>0</v>
@@ -20730,7 +20646,7 @@
     </row>
     <row r="4" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B4">
         <v>0</v>
@@ -20828,7 +20744,7 @@
     </row>
     <row r="5" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B5">
         <v>0</v>
@@ -20926,7 +20842,7 @@
     </row>
     <row r="6" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B6">
         <f>B2</f>
@@ -21055,7 +20971,7 @@
     </row>
     <row r="7" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B7">
         <v>0</v>
@@ -21153,7 +21069,7 @@
     </row>
     <row r="8" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B8">
         <f>B2</f>
@@ -21286,21 +21202,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101002041A8AB53924247A2770D65450F5227" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="90fff4f083191fe75a03dbd50c7739fc">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="1659011e-6b88-4225-9a61-aaf33aaf19e8" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="7fee88694a371868130ae0617c69143c" ns2:_="">
     <xsd:import namespace="1659011e-6b88-4225-9a61-aaf33aaf19e8"/>
@@ -21444,24 +21345,22 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{17260655-F13F-478B-A86E-BECC747CF292}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0D4397E7-5A43-4CB6-BF99-134960B037B4}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{54267EE1-F0B7-41A6-A9FD-F939C48C67EC}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -21477,4 +21376,21 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0D4397E7-5A43-4CB6-BF99-134960B037B4}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{17260655-F13F-478B-A86E-BECC747CF292}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>